<commit_message>
Paso 3: columna coleccion, 16 preguntas en borrador (climático y bioseguridad) y Recall@5 por colección
</commit_message>
<xml_diff>
--- a/corpus/md/para_investigacion.xlsx
+++ b/corpus/md/para_investigacion.xlsx
@@ -421,7 +421,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Para revisar por Investigación (generado el 2026-10-15 02:34)</t>
+          <t>Para revisar por Investigación (generado el 2026-10-15 03:07)</t>
         </is>
       </c>
     </row>
@@ -5810,31 +5810,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>coleccion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>pregunta</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>doc_esperado_actual</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>top5_hoy_en_diagnostico_md</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>nota</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>top5_hoy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>docs_aceptables (completar, separados por ;)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>comentario (completar)</t>
         </is>
@@ -5843,230 +5853,814 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>¿Qué medidas contempla el plan de contingencia del SAG ante un brote de influenza aviar en Chile?</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | D25: Evaluation of three commercially available influenza A type specific blocking EL</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | D-PM284: Active surveillance of avian influenza in the southwestern Poyang Lake area, Chi</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>¿Qué pruebas recomienda la OMSA para diagnosticar la influenza aviar altamente patógena?</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>D-PM159: The role of artificial intelligence in detecting avian influenza virus outbreaks | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | D25: Evaluation of three commercially available influenza A type specific blocking EL</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D8</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>D-PM159: The role of artificial intelligence in detecting avian influenza virus outbreaks | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | D-PM022: Serologic Evidence of Occupational Exposure to Avian Influenza Viruses at the Wi</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>¿Cómo diagnostica el SAG la influenza aviar con ELISA y RT-PCR en tiempo real?</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>D22</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D22</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t xml:space="preserve">D-PM366: Development and Analytical Validation of a Multiplex Real-Time RT-PCR Assay for  | D-PM159: The role of artificial intelligence in detecting avian influenza virus outbreaks | D-PM179: Statistical Analysis of the Performance of Local Veterinary Laboratories in Mole | D-PM028: Distribution of avian influenza viruses according to environmental surveillance  | D-PM169: Redesign and Validation of a Real-Time RT-PCR to Improve Surveillance for Avian </t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>¿Cómo se toman muestras de aves para detectar influenza A y enfermedad de Newcastle?</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>D27</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D27</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>D27: Avian Sample Collection for Influenza A and Newcastle Disease (NVSL-WI-0023) | D-PM022: Serologic Evidence of Occupational Exposure to Avian Influenza Viruses at the Wi | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>¿Qué ensayo de RT-PCR en tiempo real detecta influenza tipo A y los subtipos H5 y H7?</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>D33</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D33</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>D-PM028: Distribution of avian influenza viruses according to environmental surveillance  | D-PM170: High number of HPAI H5 virus infections and antibodies in wild carnivores in the | D-PM169: Redesign and Validation of a Real-Time RT-PCR to Improve Surveillance for Avian  | D-PM307: Molecular Detection and Genetic Characterization of H9N2 Avian Influenza Virus i | D-PM176: Environmental monitoring and spatiotemporal trend analysis of avian influenza vi</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>¿Se puede usar sangre en tiras de papel filtro en vez de suero para detectar anticuerpos de influenza aviar en aves silvestres?</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>D23</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D23</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>D23: Comparison of whole blood on filter strips with serum for avian influenza virus  | D24: Surveillance of live birds for active and past infections reveals the impact of  | D-PM022: Serologic Evidence of Occupational Exposure to Avian Influenza Viruses at the Wi | D-PM347: Serological Evidence of Flavivirus Exposure and Limited Avian Influenza Exposure</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>¿Qué impacto tuvo el H5N1 altamente patógeno en las poblaciones de aves marinas?</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>D24</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D24</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>D24: Surveillance of live birds for active and past infections reveals the impact of  | D-PM305: Genomic detection of highly pathogenic avian influenza H5N1 in Antarctic seabird | D-PM127: Serological analysis in humans in Malaysian Borneo suggests prior exposure to H5</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>¿Qué kit ELISA de IDEXX detecta anticuerpos contra influenza aviar?</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>D20</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D20 (D11 también nombra el kit)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>D8: Manual Terrestre de la OMSA, Capitulo 3.3.4: Influenza aviar (incluida la infecc | D-PM112: Vaccination of poultry against highly pathogenic avian influenza – Part 2. Surve | D-PM022: Serologic Evidence of Occupational Exposure to Avian Influenza Viruses at the Wi | D-PM300: Age-related serological response to H9N2 infection in southwest Tripoli, Libya</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>¿Qué kits comerciales aprueba el SAG para diagnosticar influenza aviar?</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>D11</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D11</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>D8: Manual Terrestre de la OMSA, Capitulo 3.3.4: Influenza aviar (incluida la infecc | D-PM112: Vaccination of poultry against highly pathogenic avian influenza – Part 2. Surve | D-PM366: Development and Analytical Validation of a Multiplex Real-Time RT-PCR Assay for  | D-PM159: The role of artificial intelligence in detecting avian influenza virus outbreaks | D-PM347: Serological Evidence of Flavivirus Exposure and Limited Avian Influenza Exposure</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>¿Cómo se recolectan, envían y almacenan las muestras para diagnóstico?</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D10</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>D10: Codes and Manuals: Terrestrial Manual, Capitulo 1.1.2 Collection, submission and | D5: Guia sobre la reglamentacion relativa al transporte de sustancias infecciosas 20 | D22: Instructivo Tecnico para el Diagnostico de Influenza Aviar mediante ELISA y RT-P</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>¿Cómo se valida una prueba de diagnóstico de enfermedades infecciosas en animales?</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D7</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>D7: Manual Terrestre de la OMSA, Capitulo 1.1.6: Validacion de las pruebas de diagno | D6: Manual Terrestre de la OMSA, Capitulo 1.1.5: Gestion de calidad en los laborator | D10: Codes and Manuals: Terrestrial Manual, Capitulo 1.1.2 Collection, submission and | D19: Manual Terrestre de la OMSA, Capitulo 2.2.1: Desarrollo y optimizacion de los en</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>diagnostico_md</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>¿Qué información mínima hay que reportar en un experimento de PCR cuantitativa en tiempo real?</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>D32</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación; sale del título de D32</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>D32: MIQE 2.0: Revision of the Minimum Information for Publication of Quantitative Re</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>¿Cómo se dispersa el virus de la influenza aviar por el viento desde granjas avícolas con brotes?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A2;CLI-131</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>A2: Wind-Mediated Spread of Low-Pathogenic Avian Influenza Virus into the Environmen | CLI-024: Predicting highly pathogenic avian influenza H5N1 outbreak risk using extreme we | CLI-004: Disentangling the role of poultry farms and wild birds in the spread of highly p</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>¿Qué factores explicaron la dinámica espacio-temporal de la influenza aviar H5N1 en Chile?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A4;CLI-020</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>A4: Spatio-temporal dynamics and drivers of highly pathogenic avian influenza H5N1 i | CLI-085: Environmental factors and spatiotemporal distribution characteristics of the glo | CLI-020: Transboundary Spread and Ecological Drivers of HPAI H5N1 Clade 2.3.4.4b During t</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>¿Qué papel tuvieron las aves silvestres en la panzootia mundial de influenza aviar H5 entre 2020 y 2023?</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CLI-017</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4: Spatio-temporal dynamics and drivers of highly pathogenic avian influenza H5N1 i | CLI-017: The role of wild birds in the global highly pathogenic avian influenza H5 panzoo | CLI-024: Predicting highly pathogenic avian influenza H5N1 outbreak risk using extreme we | CLI-133: Mitigating Risk: Predicting H5N1 Avian Influenza Spread with an Empirical Model </t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>¿Cómo influyen la lluvia y las aves silvestres en los brotes de influenza aviar en aves de corral de Australia?</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CLI-009</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CLI-009: Rainfall driven and wild-bird mediated avian influenza virus outbreaks in Austra | CLI-001: Avian Influenza in Wild Birds and Poultry: Dissemination Pathways, Monitoring Me | CLI-083: Landscape effects and spatial patterns of avian influenza virus in Danish wild b | CLI-006: Transmission dynamics of highly pathogenic avian influenza among multiple waterf</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>¿Se pueden predecir brotes de H5N1 con datos de clima extremo y de migración de aves?</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CLI-024</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CLI-106: Spatio-temporal Modelling of H5N1 Avian Influenza Outbreaks in Europe (2021-2024 | CLI-024: Predicting highly pathogenic avian influenza H5N1 outbreak risk using extreme we | A4: Spatio-temporal dynamics and drivers of highly pathogenic avian influenza H5N1 i</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>¿Qué relación hay entre los brotes de influenza aviar altamente patógena y las condiciones meteorológicas en Japón?</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CLI-064</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CLI-064: Association between highly pathogenic avian influenza outbreaks and weather cond | CLI-104: Avian Influenza at the Wild Bird–Poultry Interface: An Asia-Focused Review with  | CLI-053: Potential risk zones and climatic factors influencing the occurrence and persist</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>¿Cómo cambia el calentamiento climático el impacto de la influenza aviar altamente patógena?</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CLI-098</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CLI-098: Host responses and viral traits interact to shape the impacts of climate warming | CLI-024: Predicting highly pathogenic avian influenza H5N1 outbreak risk using extreme we | CLI-016: Avian Influenza: Lessons from Past Outbreaks and an Inventory of Data Sources, M | CLI-064: Association between highly pathogenic avian influenza outbreaks and weather cond</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>climatico_md</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>¿Cómo se usan muestreadores pasivos para vigilar virus de influenza aviar en humedales?</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CLI-087</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>CLI-087: Exploring the Use of Passive Samplers for the Surveillance of Avian Influenza Vi | CLI-003: Highly Pathogenic Avian Influenza Viruses at the Wild–Domestic Bird Interface in | CLI-070: Recurring Trans-Atlantic Incursion of Clade 2.3.4.4b H5N1 Viruses by Long Distan | CLI-020: Transboundary Spread and Ecological Drivers of HPAI H5N1 Clade 2.3.4.4b During t | CLI-125: Monitoring influenza A virus in wild migratory birds and waterfowl in Libya usin</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>¿Qué tan eficaz es la limpieza y desinfección de vehículos y jaulas de transporte frente a la influenza aviar?</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BIO-009</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BIO-009: Avian influenza outbreaks: evaluating the efficacy of cleaning and disinfection  | BIO-046: Risk Areas for Influenza A(H5) Environmental Contamination in Live Bird Markets, | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar | F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de </t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>¿Qué fallas de bioseguridad se encontraron en granjas avícolas afectadas por influenza aviar altamente patógena?</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BIO-041;BIO-028</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BIO-052: Avian influenza spillover into poultry: environmental influences and biosecurity | BIO-074: Risk Factors Associated with Avian Influenza Subtype H9 Outbreaks in Poultry Far | BIO-031: Assessment of biosecurity practices and risk factors for avian influenza outbrea | BIO-004: Monitoring biosecurity in poultry production: an overview of databases reporting | BIO-040: Clustering broiler farmers based on their behavioural differences towards biosec</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>¿Qué medidas contempla el plan de contingencia del SAG para la influenza aviar?</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>F1;E7</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | C30: Recomendacion del CAVEI sobre incorporacion de la vacunacion contra influenza av</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>¿Cómo se compostan las aves muertas durante la respuesta a un brote de influenza aviar altamente patógena?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar | C5: Avian Influenza: informacion general y medidas de prevencion (ficha tecnica ofic | C28: Gripe aviar y otras gripes de origen zoonotico (nota descriptiva)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>¿Cómo se despuebla a gallinas ponedoras enjauladas usando espuma con dióxido de carbono y nitrógeno?</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>C11: Carbon dioxide and nitrogen infused compressed air foam for depopulation of cage | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>¿Qué medidas de bioseguridad deben seguir las personas en una emergencia zoosanitaria por influenza aviar?</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>E5: Instructivo Técnico – Bioseguridad de las Personas en una Emergencia Zoosanitari | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | BIO-057: Preparedness, prevention and control related to zoonotic avian influenza</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>¿Qué niveles de mortalidad permiten sospechar influenza aviar en gallinas ponedoras?</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>C17;C18</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BIO-068: Risk factors for avian influenza in Danish poultry and wild birds during the epi | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar | C18: Mortality levels and production indicators for suspicion of highly pathogenic av | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | E7: Procedimiento P-PP-VE-006 – Contingencia de Influenza Aviar</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>bioseguridad_md</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>¿Qué factores de riesgo hubo para la introducción de H5N1 en granjas comerciales de pavos en Estados Unidos?</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BIO-054</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>borrador, falta validar con Investigación</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BIO-037: Risk Factors for Introduction of H5N1 Highly Pathogenic Avian Influenza Virus in | BIO-025: Farm-Level Risk Factors Associated With Avian Influenza A (H5) and A (H9) Flock- | BIO-068: Risk factors for avian influenza in Danish poultry and wild birds during the epi | C6: Farm biosecurity practices affecting avian influenza virus circulation in commer | BIO-019: An assessment of the highly pathogenic avian influenza resurgence at human-poult</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Lista para Investigación actualizada (incluye BIO-123, BIO-126 y BIO-138)
</commit_message>
<xml_diff>
--- a/corpus/md/para_investigacion.xlsx
+++ b/corpus/md/para_investigacion.xlsx
@@ -421,7 +421,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Para revisar por Investigación (generado el 2026-10-15 03:07)</t>
+          <t>Para revisar por Investigación (generado el 2026-10-15 03:30)</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -498,7 +498,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
@@ -684,10 +684,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C13" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D13" t="n">
         <v>32</v>
@@ -696,7 +696,7 @@
         <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2312,7 +2312,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BIO-011</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2322,27 +2322,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Con pago</t>
+          <t>Caído</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Machine learning-driven dynamic risk prediction for highly pathogenic avian influenza at poultry farms in Republic of Korea: Daily risk estimation for individual premises</t>
+          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/tbed.14419</t>
+          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>OpenAlex: sin acceso abierto (is_oa = false)</t>
+          <t>d) PDF directo: sin respuesta en 10 s</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Buscar versión libre (repositorio del autor) o conseguir el PDF.</t>
+          <t>Revisar si la URL sigue viva o buscar otra.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2354,7 +2354,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BIO-023</t>
+          <t>BIO-011</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>The Impact of Experiences and Perceptions of Highly Pathogenic Avian Influenza (HPAI) on Water‐Related Biosecurity Behaviour in Rural Vietnam</t>
+          <t>Machine learning-driven dynamic risk prediction for highly pathogenic avian influenza at poultry farms in Republic of Korea: Daily risk estimation for individual premises</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/risa.13753</t>
+          <t>https://doi.org/10.1111/tbed.14419</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2396,7 +2396,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BIO-027</t>
+          <t>BIO-023</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2411,12 +2411,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Analysis of the movement of live broilers in Guangxi, China and implications for avian influenza control</t>
+          <t>The Impact of Experiences and Perceptions of Highly Pathogenic Avian Influenza (HPAI) on Water‐Related Biosecurity Behaviour in Rural Vietnam</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/tbed.14351</t>
+          <t>https://doi.org/10.1111/risa.13753</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BIO-045</t>
+          <t>BIO-027</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2453,12 +2453,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Characterization of practices influencing avian influenza virus transmission risk in live bird markets in Northern Vietnam</t>
+          <t>Analysis of the movement of live broilers in Guangxi, China and implications for avian influenza control</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.prevetmed.2026.106958</t>
+          <t>https://doi.org/10.1111/tbed.14351</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BIO-053</t>
+          <t>BIO-045</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2495,12 +2495,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>A case-control study of the infection risk of H5N8 highly pathogenic avian influenza in Japan during the winter of 2020–2021</t>
+          <t>Characterization of practices influencing avian influenza virus transmission risk in live bird markets in Northern Vietnam</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.rvsc.2024.105149</t>
+          <t>https://doi.org/10.1016/j.prevetmed.2026.106958</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2522,7 +2522,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BIO-055</t>
+          <t>BIO-053</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2537,12 +2537,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Preventive effect of on-farm biosecurity practices against highly pathogenic avian influenza (HPAI) H5N6 infection on commercial layer farms in the Republic of Korea during the 2016-17 epidemic: A case-control study</t>
+          <t>A case-control study of the infection risk of H5N8 highly pathogenic avian influenza in Japan during the winter of 2020–2021</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.prevetmed.2021.105556</t>
+          <t>https://doi.org/10.1016/j.rvsc.2024.105149</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2564,7 +2564,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BIO-078</t>
+          <t>BIO-055</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2579,12 +2579,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Prevalence and risk factors of Avian Influenza Viruses among household ducks in Chattogram, Bangladesh</t>
+          <t>Preventive effect of on-farm biosecurity practices against highly pathogenic avian influenza (HPAI) H5N6 infection on commercial layer farms in the Republic of Korea during the 2016-17 epidemic: A case-control study</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s11259-021-09874-4</t>
+          <t>https://doi.org/10.1016/j.prevetmed.2021.105556</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2606,12 +2606,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>A14</t>
+          <t>BIO-078</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2621,12 +2621,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Acute synergistic effects of air temperature, humidity, and velocity on homeostasis of market-size broilers</t>
+          <t>Prevalence and risk factors of Avian Influenza Viruses among household ducks in Chattogram, Bangladesh</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://doi.org/10.13031/2013.12971</t>
+          <t>https://doi.org/10.1007/s11259-021-09874-4</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2648,7 +2648,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CLI-055</t>
+          <t>A14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2663,12 +2663,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Spatiotemporal risk assessment for avian influenza outbreak based on the dynamics of habitat suitability for wild birds.</t>
+          <t>Acute synergistic effects of air temperature, humidity, and velocity on homeostasis of market-size broilers</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/tbed.14376</t>
+          <t>https://doi.org/10.13031/2013.12971</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2690,7 +2690,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CLI-056</t>
+          <t>CLI-055</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2705,12 +2705,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Airborne Avian Influenza Virus in Ambient Air in the Winter Habitats of Migratory Birds.</t>
+          <t>Spatiotemporal risk assessment for avian influenza outbreak based on the dynamics of habitat suitability for wild birds.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1021/acs.est.2c04528</t>
+          <t>https://doi.org/10.1111/tbed.14376</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2732,7 +2732,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CLI-066</t>
+          <t>CLI-056</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2747,12 +2747,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Wild Birds Affected by Highly Pathogenic Avian Influenza A (H5N1) Worldwide: Epidemiological Insights Into the Recent Panzootic.</t>
+          <t>Airborne Avian Influenza Virus in Ambient Air in the Winter Habitats of Migratory Birds.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/gcb.70523</t>
+          <t>https://doi.org/10.1021/acs.est.2c04528</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2774,7 +2774,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CLI-075</t>
+          <t>CLI-066</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2789,12 +2789,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Distinct but connected avian influenza virus activities in wetlands and live poultry markets in Bangladesh, 2018-2019.</t>
+          <t>Wild Birds Affected by Highly Pathogenic Avian Influenza A (H5N1) Worldwide: Epidemiological Insights Into the Recent Panzootic.</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/tbed.14450</t>
+          <t>https://doi.org/10.1111/gcb.70523</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2816,7 +2816,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CLI-091</t>
+          <t>CLI-075</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2831,12 +2831,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Ecology of avian influenza viruses in migratory birds wintering within the Yangtze River wetlands.</t>
+          <t>Distinct but connected avian influenza virus activities in wetlands and live poultry markets in Bangladesh, 2018-2019.</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.scib.2021.03.023</t>
+          <t>https://doi.org/10.1111/tbed.14450</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2858,7 +2858,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CLI-100</t>
+          <t>CLI-091</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2873,12 +2873,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Assessment of the spatiotemporal risk of avian influenza between waterfowl and poultry farms during the annual cycle: A spatial prediction study focused on seasonal distribution changes in resident waterfowl in South Korea.</t>
+          <t>Ecology of avian influenza viruses in migratory birds wintering within the Yangtze River wetlands.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/tbed.14669</t>
+          <t>https://doi.org/10.1016/j.scib.2021.03.023</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2900,7 +2900,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CLI-114</t>
+          <t>CLI-100</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Estimation of Avian Influenza Viruses in Water Environments of Live Poultry Markets in Changsha, China, 2014 to 2018.</t>
+          <t>Assessment of the spatiotemporal risk of avian influenza between waterfowl and poultry farms during the annual cycle: A spatial prediction study focused on seasonal distribution changes in resident waterfowl in South Korea.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s12560-021-09506-9</t>
+          <t>https://doi.org/10.1111/tbed.14669</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2942,7 +2942,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CLI-116</t>
+          <t>CLI-114</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2957,12 +2957,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Detection by environmental surveillance and genomic characterization of H5N8 highly pathogenic avian influenza virus from a poultry meat market in Beijing, China, 2021-22.</t>
+          <t>Estimation of Avian Influenza Viruses in Water Environments of Live Poultry Markets in Changsha, China, 2014 to 2018.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s11259-022-10005-w</t>
+          <t>https://doi.org/10.1007/s12560-021-09506-9</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2984,7 +2984,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CLI-128</t>
+          <t>CLI-116</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2999,12 +2999,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Predator-Prey Trophic Interactions and Seasonality of Highly Pathogenic Avian Influenza Virus in Denmark, 2016-2023.</t>
+          <t>Detection by environmental surveillance and genomic characterization of H5N8 highly pathogenic avian influenza virus from a poultry meat market in Beijing, China, 2021-22.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/zph.70019</t>
+          <t>https://doi.org/10.1007/s11259-022-10005-w</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3026,12 +3026,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>D-PM007</t>
+          <t>CLI-128</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3041,12 +3041,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>H7N9 influenza virus surveillance in Gansu, China in 2017.</t>
+          <t>Predator-Prey Trophic Interactions and Seasonality of Highly Pathogenic Avian Influenza Virus in Denmark, 2016-2023.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.virusres.2021.198335</t>
+          <t>https://doi.org/10.1111/zph.70019</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3068,7 +3068,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>D-PM045</t>
+          <t>D-PM007</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3083,12 +3083,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Surveillance of multiple subtype specific antibodies against avian influenza viruses among egg yolk in wild ducks from northeast China, 2017-2019.</t>
+          <t>H7N9 influenza virus surveillance in Gansu, China in 2017.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.micpath.2020.104618</t>
+          <t>https://doi.org/10.1016/j.virusres.2021.198335</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -3110,7 +3110,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>D-PM049</t>
+          <t>D-PM045</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3125,12 +3125,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Molecular Detection of Avian Influenza Virus in Wild Birds in Morocco, 2016-2019.</t>
+          <t>Surveillance of multiple subtype specific antibodies against avian influenza viruses among egg yolk in wild ducks from northeast China, 2017-2019.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1637/aviandiseases-D-21-00070</t>
+          <t>https://doi.org/10.1016/j.micpath.2020.104618</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -3152,7 +3152,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>D-PM118</t>
+          <t>D-PM049</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3167,12 +3167,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Surveillance and Sequestration Strategies to Reduce the Likelihood of Transporting Highly Pathogenic Avian Influenza Virus Contaminated Layer Manure.</t>
+          <t>Molecular Detection of Avian Influenza Virus in Wild Birds in Morocco, 2016-2019.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1637/0005-2086-65.2.219</t>
+          <t>https://doi.org/10.1637/aviandiseases-D-21-00070</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -3194,7 +3194,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>D-PM199</t>
+          <t>D-PM118</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3209,12 +3209,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Development of a Novel Korean H9-Specific rRT-PCR Assay and Its Application for Avian Influenza Virus Surveillance in Korea.</t>
+          <t>Surveillance and Sequestration Strategies to Reduce the Likelihood of Transporting Highly Pathogenic Avian Influenza Virus Contaminated Layer Manure.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s12275-023-00088-8</t>
+          <t>https://doi.org/10.1637/0005-2086-65.2.219</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -3236,7 +3236,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>D-PM204</t>
+          <t>D-PM199</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3251,12 +3251,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Molecular diagnostics in clinical microbiology: Advances, applications, and future directions.</t>
+          <t>Development of a Novel Korean H9-Specific rRT-PCR Assay and Its Application for Avian Influenza Virus Surveillance in Korea.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.diagmicrobio.2025.117223</t>
+          <t>https://doi.org/10.1007/s12275-023-00088-8</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3278,7 +3278,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>D-PM255</t>
+          <t>D-PM204</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3293,12 +3293,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Active Surveillance and Genetic Characterization of Prevalent Velogenic Newcastle Disease and Highly Pathogenic Avian Influenza H5N8 Viruses Among Migratory Wild Birds in Southern Egypt During 2015-2018.</t>
+          <t>Molecular diagnostics in clinical microbiology: Advances, applications, and future directions.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s12560-022-09532-1</t>
+          <t>https://doi.org/10.1016/j.diagmicrobio.2025.117223</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -3320,7 +3320,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>D-PM353</t>
+          <t>D-PM255</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3335,12 +3335,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Four-season bulk tank milk surveillance for brucellosis, influenza A virus, and Q fever in Korean dairy farms.</t>
+          <t>Active Surveillance and Genetic Characterization of Prevalent Velogenic Newcastle Disease and Highly Pathogenic Avian Influenza H5N8 Viruses Among Migratory Wild Birds in Southern Egypt During 2015-2018.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.rvsc.2026.106418</t>
+          <t>https://doi.org/10.1007/s12560-022-09532-1</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3362,7 +3362,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>D-PM392</t>
+          <t>D-PM353</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3377,12 +3377,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Development of an inactivated H9N2 subtype avian influenza serological DIVA vaccine using the chimeric A/B NA epitope approach.</t>
+          <t>Four-season bulk tank milk surveillance for brucellosis, influenza A virus, and Q fever in Korean dairy farms.</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.vetmic.2026.110917</t>
+          <t>https://doi.org/10.1016/j.rvsc.2026.106418</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3404,49 +3404,49 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>D-PM392</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Con pago</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Ley 18.755 – Establece normas sobre el Servicio Agrícola y Ganadero (Ley Orgánica del SAG)</t>
+          <t>Development of an inactivated H9N2 subtype avian influenza serological DIVA vaccine using the chimeric A/B NA epitope approach.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://www.bcn.cl/leychile/navegar?idNorma=30135</t>
+          <t>https://doi.org/10.1016/j.vetmic.2026.110917</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>título 46/100 y 31 palabras</t>
+          <t>OpenAlex: sin acceso abierto (is_oa = false)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>LeyChile necesita JavaScript y reCAPTCHA: bajar a mano el PDF de la norma.</t>
+          <t>Buscar versión libre (repositorio del autor) o conseguir el PDF.</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3461,17 +3461,17 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Brote Influenza aviar 2026. Antecedentes generales y situación nacional (Asesoría Técnica Parlamentaria)</t>
+          <t>Ley 18.755 – Establece normas sobre el Servicio Agrícola y Ganadero (Ley Orgánica del SAG)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://www.bcn.cl/asesoriasparlamentarias/detalle_documento.html?id=85550</t>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=30135</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>título 42/100 y 17 palabras</t>
+          <t>título 46/100 y 31 palabras</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3488,7 +3488,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3503,17 +3503,17 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Resolución Exenta N° 4.869 – Medidas sanitarias y obligaciones para terceros en contexto de enfermedades declaradas bajo control oficial</t>
+          <t>Brote Influenza aviar 2026. Antecedentes generales y situación nacional (Asesoría Técnica Parlamentaria)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://www.bcn.cl/leychile/navegar?idNorma=1224888</t>
+          <t>https://www.bcn.cl/asesoriasparlamentarias/detalle_documento.html?id=85550</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>título 41/100 y 31 palabras</t>
+          <t>título 42/100 y 17 palabras</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3530,12 +3530,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>E3</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3545,22 +3545,22 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Effect of temperature-humidity index on live performance in broiler chickens grown from 49 to 63 days of age</t>
+          <t>Resolución Exenta N° 4.869 – Medidas sanitarias y obligaciones para terceros en contexto de enfermedades declaradas bajo control oficial</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://works.bepress.com/hongwei_xin/134</t>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1224888</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>título 41/100 y 60 palabras</t>
+          <t>título 41/100 y 31 palabras</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>La URL no lleva al documento: poner el link directo o el PDF.</t>
+          <t>LeyChile necesita JavaScript y reCAPTCHA: bajar a mano el PDF de la norma.</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3572,7 +3572,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>A13</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3587,17 +3587,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Descripcion y usos de la Red de Agrometeorologia INIA (Boletin INIA N 415)</t>
+          <t>Effect of temperature-humidity index on live performance in broiler chickens grown from 49 to 63 days of age</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://sitios.inia.cl/agrometeorologia/boletin-415/</t>
+          <t>https://works.bepress.com/hongwei_xin/134</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>título 79/100 y 121 palabras</t>
+          <t>título 41/100 y 60 palabras</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3614,49 +3614,49 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BIO-001</t>
+          <t>A15</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Página equivocada</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Determinants of biosecurity practices in French duck farms after a H5N8 Highly Pathogenic Avian Influenza epidemic: The effect of farmer knowledge, attitudes and personality traits</t>
+          <t>Descripcion y usos de la Red de Agrometeorologia INIA (Boletin INIA N 415)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13462</t>
+          <t>https://sitios.inia.cl/agrometeorologia/boletin-415/</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>título 79/100 y 121 palabras</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
+          <t>La URL no lleva al documento: poner el link directo o el PDF.</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BIO-006</t>
+          <t>BIO-001</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3671,12 +3671,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Factors influencing chicken farmers' decisions to implement prevention and control measures to reduce avian influenza virus spread under endemic conditions</t>
+          <t>Determinants of biosecurity practices in French duck farms after a H5N8 Highly Pathogenic Avian Influenza epidemic: The effect of farmer knowledge, attitudes and personality traits</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13757</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13462</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3698,7 +3698,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BIO-018</t>
+          <t>BIO-006</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3713,12 +3713,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>A systematic approach to illuminate a new hot spot of avian influenza virus circulation in South Vietnam, 2016–2017</t>
+          <t>Factors influencing chicken farmers' decisions to implement prevention and control measures to reduce avian influenza virus spread under endemic conditions</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14380</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13757</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3740,7 +3740,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BIO-073</t>
+          <t>BIO-018</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3755,12 +3755,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Veterinarians' knowledge and experience of avian influenza and perspectives on control measures in the UK</t>
+          <t>A systematic approach to illuminate a new hot spot of avian influenza virus circulation in South Vietnam, 2016–2017</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/vetr.3713</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14380</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3782,7 +3782,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>BIO-073</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3797,17 +3797,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Modifications to the hemagglutinin cleavage site control the virulence of a neurotropic H1N1 influenza virus</t>
+          <t>Veterinarians' knowledge and experience of avian influenza and perspectives on control measures in the UK</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://journals.asm.org/doi/10.1128/jvi.00797-10</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/vetr.3713</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>c) Web: journals.asm.org rechaza el acceso (HTTP 403)</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3817,14 +3817,14 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3839,17 +3839,17 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Abiotic factors affecting the persistence of avian influenza virus in surface waters of waterfowl habitats</t>
+          <t>Modifications to the hemagglutinin cleavage site control the virulence of a neurotropic H1N1 influenza virus</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://aem.asm.org/content/aem/80/9/2910.full.pdf</t>
+          <t>https://journals.asm.org/doi/10.1128/jvi.00797-10</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>aem.asm.org rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: journals.asm.org rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3859,19 +3859,19 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3881,17 +3881,17 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Heat stress impairs performance and induces intestinal inflammation in broiler chickens infected with Salmonella Enteritidis</t>
+          <t>Abiotic factors affecting the persistence of avian influenza virus in surface waters of waterfowl habitats</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2012.709315?needAccess=true&amp;role=button</t>
+          <t>https://aem.asm.org/content/aem/80/9/2910.full.pdf</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>www.tandfonline.com rechaza el acceso (HTTP 403)</t>
+          <t>aem.asm.org rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3908,7 +3908,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3923,12 +3923,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Inactivation of the infectivity of two highly pathogenic avian influenza viruses and a virulent Newcastle disease virus by ultraviolet radiation</t>
+          <t>Heat stress impairs performance and induces intestinal inflammation in broiler chickens infected with Salmonella Enteritidis</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2013.853867?needAccess=true&amp;role=button</t>
+          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2012.709315?needAccess=true&amp;role=button</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3950,7 +3950,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CLI-005</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3965,17 +3965,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Determinants of highly pathogenic avian influenza spread during bird migration</t>
+          <t>Inactivation of the infectivity of two highly pathogenic avian influenza viruses and a virulent Newcastle disease virus by ultraviolet radiation</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1098/rsos.260182</t>
+          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2013.853867?needAccess=true&amp;role=button</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>c) Web: royalsocietypublishing.org rechaza el acceso (HTTP 403)</t>
+          <t>www.tandfonline.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3985,14 +3985,14 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CLI-023</t>
+          <t>CLI-005</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4007,17 +4007,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>A threat from both sides: Multiple introductions of genetically distinct H5 HPAI viruses into Canada via both East Asia-Australasia/Pacific and Atlantic flyways.</t>
+          <t>Determinants of highly pathogenic avian influenza spread during bird migration</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1093/ve/veac077</t>
+          <t>https://doi.org/10.1098/rsos.260182</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>c) Web: academic.oup.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: royalsocietypublishing.org rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4034,7 +4034,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CLI-043</t>
+          <t>CLI-023</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4049,17 +4049,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Global dissemination of influenza A virus is driven by wild bird migration through arctic and subarctic zones.</t>
+          <t>A threat from both sides: Multiple introductions of genetically distinct H5 HPAI viruses into Canada via both East Asia-Australasia/Pacific and Atlantic flyways.</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://www.authorea.com/doi/pdf/10.22541/au.164372348.88612449</t>
+          <t>https://doi.org/10.1093/ve/veac077</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>www.authorea.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: academic.oup.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4069,14 +4069,14 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CLI-059</t>
+          <t>CLI-043</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4091,17 +4091,17 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Waterfowl show spatiotemporal trends in influenza A H5 and H7 infections but limited taxonomic variation.</t>
+          <t>Global dissemination of influenza A virus is driven by wild bird migration through arctic and subarctic zones.</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/eap.2906</t>
+          <t>https://www.authorea.com/doi/pdf/10.22541/au.164372348.88612449</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>www.authorea.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4118,7 +4118,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CLI-061</t>
+          <t>CLI-059</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4133,17 +4133,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Seasonality of influenza and coseasonality with avian influenza in Bangladesh, 2010-19: a retrospective, time-series analysis.</t>
+          <t>Waterfowl show spatiotemporal trends in influenza A H5 and H7 infections but limited taxonomic variation.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>http://www.thelancet.com/article/S2214109X22002121/pdf</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/eap.2906</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4160,7 +4160,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CLI-068</t>
+          <t>CLI-061</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4175,17 +4175,17 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Improved method for avian influenza virus isolation from environmental water samples.</t>
+          <t>Seasonality of influenza and coseasonality with avian influenza in Bangladesh, 2010-19: a retrospective, time-series analysis.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14639</t>
+          <t>http://www.thelancet.com/article/S2214109X22002121/pdf</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4202,7 +4202,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CLI-090</t>
+          <t>CLI-068</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4217,17 +4217,17 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Spatiotemporal patterns of low and highly pathogenic avian influenza virus prevalence in murres in Canada from 2007 to 2022—a case study for wildlife viral monitoring</t>
+          <t>Improved method for avian influenza virus isolation from environmental water samples.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1139/facets-2023-0185</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14639</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>c) Web: www.facetsjournal.com rechaza el acceso (HTTP 403)</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4237,14 +4237,14 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CLI-119</t>
+          <t>CLI-090</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4259,17 +4259,17 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Cost of migration increased during an outbreak of highly pathogenic avian influenza virus</t>
+          <t>Spatiotemporal patterns of low and highly pathogenic avian influenza virus prevalence in murres in Canada from 2007 to 2022—a case study for wildlife viral monitoring</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/jav.03616</t>
+          <t>https://doi.org/10.1139/facets-2023-0185</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>c) Web: nsojournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: www.facetsjournal.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4286,7 +4286,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CLI-130</t>
+          <t>CLI-119</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4301,17 +4301,17 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Integrating wild bird and environmental samples can strengthen avian influenza surveillance</t>
+          <t>Cost of migration increased during an outbreak of highly pathogenic avian influenza virus</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/1365-2664.70584</t>
+          <t>https://doi.org/10.1002/jav.03616</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>c) Web: besjournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: nsojournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4328,12 +4328,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>D-PM110</t>
+          <t>CLI-130</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4343,17 +4343,17 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Surveillance of avian influenza viruses in Hebei Province of China from 2021 to 2023: Identification of a novel reassortant H3N3.</t>
+          <t>Integrating wild bird and environmental samples can strengthen avian influenza surveillance</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://www.journalofinfection.com/article/S0163-4453(24)00174-9/pdf</t>
+          <t>https://doi.org/10.1111/1365-2664.70584</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>www.journalofinfection.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: besjournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4363,14 +4363,14 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>D-PM139</t>
+          <t>D-PM110</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4385,17 +4385,17 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Wastewater monitoring of human and avian influenza A viruses in Northern Ireland: a genomic surveillance study.</t>
+          <t>Surveillance of avian influenza viruses in Hebei Province of China from 2021 to 2023: Identification of a novel reassortant H3N3.</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>http://www.thelancet.com/article/S2666524724001757/pdf</t>
+          <t>https://www.journalofinfection.com/article/S0163-4453(24)00174-9/pdf</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
+          <t>www.journalofinfection.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4412,7 +4412,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>D-PM139</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4427,17 +4427,17 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>The MIQE Guidelines: Minimum Information for Publication of Quantitative Real-Time PCR Experiments</t>
+          <t>Wastewater monitoring of human and avian influenza A viruses in Northern Ireland: a genomic surveillance study.</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>http://clinchem.aaccjnls.org/content/clinchem/55/4/611.full.pdf</t>
+          <t>http://www.thelancet.com/article/S2666524724001757/pdf</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>academic.oup.com rechaza el acceso (HTTP 403)</t>
+          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4454,49 +4454,49 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
+          <t>The MIQE Guidelines: Minimum Information for Publication of Quantitative Real-Time PCR Experiments</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
+          <t>http://clinchem.aaccjnls.org/content/clinchem/55/4/611.full.pdf</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>título 69/100 (&lt; 80) y 1083 palabras</t>
+          <t>academic.oup.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Abrir el .md y confirmar que es el documento correcto.</t>
+          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4511,17 +4511,17 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Codigo Sanitario para los Animales Terrestres, Capitulo 1.1: Notificacion de enfermedades y presentacion de datos epidemiologicos (articulo 1.1.3)</t>
+          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://www.woah.org/fileadmin/Home/eng/Health_standards/tahc/2023/chapitre_notification.pdf</t>
+          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>título 58/100 (&lt; 80) y 1108 palabras</t>
+          <t>título 69/100 (&lt; 80) y 1083 palabras</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4538,7 +4538,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4553,17 +4553,17 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>SAG logra en tiempo record la reapertura de los principales mercados de productos avicolas tras foco de influenza aviar (comunicado)</t>
+          <t>Codigo Sanitario para los Animales Terrestres, Capitulo 1.1: Notificacion de enfermedades y presentacion de datos epidemiologicos (articulo 1.1.3)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/noticias/sag-logra-en-tiempo-record-la-reapertura-de-los-principales-mercados-de-productos-avicolas-tras-foco-de-influenza-aviar</t>
+          <t>https://www.woah.org/fileadmin/Home/eng/Health_standards/tahc/2023/chapitre_notification.pdf</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>título 53/100 (&lt; 80) y 431 palabras</t>
+          <t>título 58/100 (&lt; 80) y 1108 palabras</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4580,7 +4580,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>C33</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4595,17 +4595,17 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Chile se autodeclara pais libre de influenza aviar altamente patogena en aves de corral (comunicado)</t>
+          <t>SAG logra en tiempo record la reapertura de los principales mercados de productos avicolas tras foco de influenza aviar (comunicado)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/noticias/chile-se-autodeclara-pais-libre-de-influenza-aviar-altamente-patogena-en-aves-de-corral</t>
+          <t>https://www.sag.gob.cl/noticias/sag-logra-en-tiempo-record-la-reapertura-de-los-principales-mercados-de-productos-avicolas-tras-foco-de-influenza-aviar</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>título 70/100 (&lt; 80) y 717 palabras</t>
+          <t>título 53/100 (&lt; 80) y 431 palabras</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4622,7 +4622,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4637,17 +4637,17 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>SAG – Pecuaria (ámbito de acción)</t>
+          <t>Chile se autodeclara pais libre de influenza aviar altamente patogena en aves de corral (comunicado)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/ambitos-de-accion/pecuaria</t>
+          <t>https://www.sag.gob.cl/noticias/chile-se-autodeclara-pais-libre-de-influenza-aviar-altamente-patogena-en-aves-de-corral</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>título 59/100 (&lt; 80) y 487 palabras</t>
+          <t>título 70/100 (&lt; 80) y 717 palabras</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4664,7 +4664,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>E19</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4679,17 +4679,17 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>SAG – Resolución Exenta N° 7.050: aprueba Instructivo Técnico de Bioseguridad de las Personas (influenza aviar), versión 3</t>
+          <t>SAG – Pecuaria (ámbito de acción)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/content/aprueba-instructivo-tecnico-de-bioseguridad-de-las-personas-en-una-emergencia-zoosanitaria-con-riesgo-de-zoonosis-influenza-aviar-ia-version-3-y-dejese-sin-efecto-la-resolucion-exenta-ndeg-39962026</t>
+          <t>https://www.sag.gob.cl/ambitos-de-accion/pecuaria</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>título 79/100 (&lt; 80) y 339 palabras</t>
+          <t>título 59/100 (&lt; 80) y 487 palabras</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4706,7 +4706,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>E21</t>
+          <t>E19</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4721,17 +4721,17 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>FAO – EMPRES-i (página 'Acerca de' del sitio data.apps.fao.org)</t>
+          <t>SAG – Resolución Exenta N° 7.050: aprueba Instructivo Técnico de Bioseguridad de las Personas (influenza aviar), versión 3</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://data.apps.fao.org/static/sites/empres-i/about.html</t>
+          <t>https://www.sag.gob.cl/content/aprueba-instructivo-tecnico-de-bioseguridad-de-las-personas-en-una-emergencia-zoosanitaria-con-riesgo-de-zoonosis-influenza-aviar-ia-version-3-y-dejese-sin-efecto-la-resolucion-exenta-ndeg-39962026</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>título 56/100 (&lt; 80) y 239 palabras</t>
+          <t>título 79/100 (&lt; 80) y 339 palabras</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4748,7 +4748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>E23</t>
+          <t>E21</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4763,17 +4763,17 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>FAO – Preguntas frecuentes sobre EMA-i+ y EMPRES-i+</t>
+          <t>FAO – EMPRES-i (página 'Acerca de' del sitio data.apps.fao.org)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://www.fao.org/animal-health/resources/tools/faq-ema-i-empres-i/en</t>
+          <t>https://data.apps.fao.org/static/sites/empres-i/about.html</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>título 64/100 (&lt; 80) y 504 palabras</t>
+          <t>título 56/100 (&lt; 80) y 239 palabras</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4790,7 +4790,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>E24</t>
+          <t>E23</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4805,17 +4805,17 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>FAO – EMPRES-i (proyecto en AgroInformática)</t>
+          <t>FAO – Preguntas frecuentes sobre EMA-i+ y EMPRES-i+</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://www.fao.org/agroinformatics/projects/projects-detail/empres-i/</t>
+          <t>https://www.fao.org/animal-health/resources/tools/faq-ema-i-empres-i/en</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>título 67/100 (&lt; 80) y 242 palabras</t>
+          <t>título 64/100 (&lt; 80) y 504 palabras</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4832,12 +4832,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4847,13 +4847,17 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>IDEXX PRRS X3 Ab Test - pagina de producto</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr"/>
+          <t>FAO – EMPRES-i (proyecto en AgroInformática)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://www.fao.org/agroinformatics/projects/projects-detail/empres-i/</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>título 64/100 (&lt; 80) y 173 palabras</t>
+          <t>título 67/100 (&lt; 80) y 242 palabras</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4870,49 +4874,45 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BIO-118</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Sin ruta</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Building trustworthy generative artificial intelligence for diabetes care and limb preservation: a medical knowledge extraction case</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1177/19322968241253568</t>
-        </is>
-      </c>
+          <t>IDEXX PRRS X3 Ab Test - pagina de producto</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>solo hay la web de PMC, que no se usa (CAPTCHA); falta texto en Europe PMC</t>
+          <t>título 64/100 (&lt; 80) y 173 palabras</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Buscar el link directo al documento o el PDF.</t>
+          <t>Abrir el .md y confirmar que es el documento correcto.</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>BIO-118</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4922,44 +4922,44 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Sin texto</t>
+          <t>Sin ruta</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>PROTOCOLO DE VIGILANCIA OCUPACIONAL POR EXPOSICIÓN A INFLUENZA AVIAR Versión Nº2</t>
+          <t>Building trustworthy generative artificial intelligence for diabetes care and limb preservation: a medical knowledge extraction case</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://www.achs.cl/docs/librariesprovider2/empresa/20-gripe-aviar/legales/protocolo-de-vigilancia-ocupacional-por-exposicion-a-influenza-aviar-version-2.pdf</t>
+          <t>https://doi.org/10.1177/19322968241253568</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>no se pudo sacar texto</t>
+          <t>solo hay la web de PMC, que no se usa (CAPTCHA); falta texto en Europe PMC</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>No se pudo sacar texto: revisar el archivo.</t>
+          <t>Buscar el link directo al documento o el PDF.</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CLI-081</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4969,17 +4969,17 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>A SYSTEMATIC REVIEW AND NARRATIVE SYNTHESIS OF THE USE OF ENVIRONMENTAL SAMPLES FOR THE SURVEILLANCE OF AVIAN INFLUENZA VIRUSES IN WILD WATERBIRDS.</t>
+          <t>PROTOCOLO DE VIGILANCIA OCUPACIONAL POR EXPOSICIÓN A INFLUENZA AVIAR Versión Nº2</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-57/issue-1/JWD-D-20-00082/A-SYSTEMATIC-REVIEW-AND-NARRATIVE-SYNTHESIS-OF-THE-USE-OF/10.7589/JWD-D-20-00082.pdf</t>
+          <t>https://www.achs.cl/docs/librariesprovider2/empresa/20-gripe-aviar/legales/protocolo-de-vigilancia-ocupacional-por-exposicion-a-influenza-aviar-version-2.pdf</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>se esperaba un PDF y llegó una página web</t>
+          <t>no se pudo sacar texto</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4996,7 +4996,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CLI-105</t>
+          <t>CLI-081</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Pathogen Surveillance in Swallows (family Hirundinidae): Investigation into Role as Avian Influenza Vector in Eastern Canada Agricultural Landscapes.</t>
+          <t>A SYSTEMATIC REVIEW AND NARRATIVE SYNTHESIS OF THE USE OF ENVIRONMENTAL SAMPLES FOR THE SURVEILLANCE OF AVIAN INFLUENZA VIRUSES IN WILD WATERBIRDS.</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-60/issue-3/JWD-D-23-00167/Pathogen-Surveillance-in-Swallows-Family-Hirundinidae--Investigation-into-Role/10.7589/JWD-D-23-00167.pdf</t>
+          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-57/issue-1/JWD-D-20-00082/A-SYSTEMATIC-REVIEW-AND-NARRATIVE-SYNTHESIS-OF-THE-USE-OF/10.7589/JWD-D-20-00082.pdf</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -5038,7 +5038,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>CLI-105</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5048,77 +5048,81 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Solo resumen</t>
+          <t>Sin texto</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Genetic data and meteorological conditions: unravelling the windborne transmission of H5N1 high-pathogenicity avian influenza between commercial poultry outbreaks</t>
+          <t>Pathogen Surveillance in Swallows (family Hirundinidae): Investigation into Role as Avian Influenza Vector in Eastern Canada Agricultural Landscapes.</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://www.biorxiv.org/content/10.1101/2025.02.12.637829</t>
+          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-60/issue-3/JWD-D-23-00167/Pathogen-Surveillance-in-Swallows-Family-Hirundinidae--Investigation-into-Role/10.7589/JWD-D-23-00167.pdf</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Abstract sin Methods/Results/Discussion y 261 palabras</t>
+          <t>se esperaba un PDF y llegó una página web</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Solo llegó el resumen: conseguir el texto completo.</t>
+          <t>No se pudo sacar texto: revisar el archivo.</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>BIO-117</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr"/>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>climatico</t>
+        </is>
+      </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Tema a revisar</t>
+          <t>Solo resumen</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Answering real-world clinical questions using large language model, retrieval-augmented generation, and agentic systems</t>
+          <t>Genetic data and meteorological conditions: unravelling the windborne transmission of H5N1 high-pathogenicity avian influenza between commercial poultry outbreaks</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076251348850</t>
+          <t>https://www.biorxiv.org/content/10.1101/2025.02.12.637829</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
+          <t>Abstract sin Methods/Results/Discussion y 261 palabras</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
+          <t>Solo llegó el resumen: conseguir el texto completo.</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BIO-119</t>
+          <t>BIO-117</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -5129,12 +5133,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>From RAGs to riches: utilizing large language models to write documents for clinical trials</t>
+          <t>Answering real-world clinical questions using large language model, retrieval-augmented generation, and agentic systems</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/17407745251320806</t>
+          <t>https://doi.org/10.1177/20552076251348850</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5156,7 +5160,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>BIO-120</t>
+          <t>BIO-119</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -5167,12 +5171,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Evaluating adherence to Canadian radiology guidelines for incidental hepatobiliary findings using RAG-enabled LLMs</t>
+          <t>From RAGs to riches: utilizing large language models to write documents for clinical trials</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/08465371251323124</t>
+          <t>https://doi.org/10.1177/17407745251320806</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5194,7 +5198,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>BIO-121</t>
+          <t>BIO-120</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -5205,12 +5209,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>LLM-augmented multi-agent cooperative framework for medical case retrieval in cardiology</t>
+          <t>Evaluating adherence to Canadian radiology guidelines for incidental hepatobiliary findings using RAG-enabled LLMs</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s44443-025-00311-z</t>
+          <t>https://doi.org/10.1177/08465371251323124</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5232,7 +5236,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BIO-122</t>
+          <t>BIO-121</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -5243,12 +5247,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Performance of latest AI models, RAG, and MCP on lung cancer-related questions</t>
+          <t>LLM-augmented multi-agent cooperative framework for medical case retrieval in cardiology</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261427503</t>
+          <t>https://doi.org/10.1007/s44443-025-00311-z</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5270,7 +5274,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BIO-124</t>
+          <t>BIO-122</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -5281,12 +5285,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>A Chatbot for the Management of Bipolar Disorder: Using Retrieval-Augmented Generation With an Open-Weight Large Language Model to Answer Clinical Questions Based on the CANMAT and ISBD 2018 Guidelines for Bipolar Disorder: Un dialogueur pour la prise en charge du trouble bipolaire : utiliser la génération augmentée par récupération avec un grand modèle de langage (GML) à poids ouverts pour répondre aux questions cliniques fondées sur les lignes directrices de 2018 de CANMAT et de l'ISBD relatives au trouble bipolaire</t>
+          <t>Performance of latest AI models, RAG, and MCP on lung cancer-related questions</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/07067437261457232</t>
+          <t>https://doi.org/10.1177/20552076261427503</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5308,7 +5312,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>BIO-125</t>
+          <t>BIO-123</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -5319,12 +5323,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Development of a cancer information chatbot model: Retrieval-augmented generation with data from the national center for cancer knowledge and information</t>
+          <t>BIOGEN: evidence-grounded multi-agent reasoning framework for transcriptomic interpretation in antimicrobial resistance</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261450314</t>
+          <t>https://doi.org/10.3389/fbinf.2026.1846404</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5346,7 +5350,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BIO-127</t>
+          <t>BIO-124</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
@@ -5357,12 +5361,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Performance and usability of retrieval-augmented large language models for stroke patient and caregiver support</t>
+          <t>A Chatbot for the Management of Bipolar Disorder: Using Retrieval-Augmented Generation With an Open-Weight Large Language Model to Answer Clinical Questions Based on the CANMAT and ISBD 2018 Guidelines for Bipolar Disorder: Un dialogueur pour la prise en charge du trouble bipolaire : utiliser la génération augmentée par récupération avec un grand modèle de langage (GML) à poids ouverts pour répondre aux questions cliniques fondées sur les lignes directrices de 2018 de CANMAT et de l'ISBD relatives au trouble bipolaire</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261464997</t>
+          <t>https://doi.org/10.1177/07067437261457232</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5384,7 +5388,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BIO-128</t>
+          <t>BIO-125</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -5395,12 +5399,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Design and multidimensional expert evaluation of a national health information portal-integrated generative AI chatbot for health literacy and awareness</t>
+          <t>Development of a cancer information chatbot model: Retrieval-augmented generation with data from the national center for cancer knowledge and information</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261481326</t>
+          <t>https://doi.org/10.1177/20552076261450314</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5422,7 +5426,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>BIO-129</t>
+          <t>BIO-126</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -5433,12 +5437,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Dynamic alignment of large language models for evidence-grounded heart failure decision support</t>
+          <t>Improved accuracy and efficiency of guideline-based orthopedic disability assessment with a retrieval-augmented AI assistant (NotebookLM) in anonymized cases</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261487568</t>
+          <t>https://doi.org/10.1177/20552076261473719</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5460,7 +5464,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>BIO-130</t>
+          <t>BIO-127</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -5471,12 +5475,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Toward an integrated animal–human nutrition intelligence via agentic retrieval-augmented language models</t>
+          <t>Performance and usability of retrieval-augmented large language models for stroke patient and caregiver support</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/fnut.2026.1815038</t>
+          <t>https://doi.org/10.1177/20552076261464997</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5498,7 +5502,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>BIO-131</t>
+          <t>BIO-128</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -5509,12 +5513,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>MEGA-RAG: a retrieval-augmented generation framework with multi-evidence guided answer refinement for mitigating hallucinations of LLMs in public health</t>
+          <t>Design and multidimensional expert evaluation of a national health information portal-integrated generative AI chatbot for health literacy and awareness</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/fpubh.2025.1635381</t>
+          <t>https://doi.org/10.1177/20552076261481326</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5536,7 +5540,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>BIO-132</t>
+          <t>BIO-129</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -5547,12 +5551,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Use of Retrieval-Augmented Large Language Model for COVID-19 Fact-Checking: Development and Usability Study</t>
+          <t>Dynamic alignment of large language models for evidence-grounded heart failure decision support</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://doi.org/10.2196/66098</t>
+          <t>https://doi.org/10.1177/20552076261487568</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5574,7 +5578,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>BIO-133</t>
+          <t>BIO-130</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
@@ -5585,12 +5589,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>GraphRAG-Vet: A Knowledge Graph-Augmented Large Language Model for Precision Bovine Disease Diagnosis</t>
+          <t>Toward an integrated animal–human nutrition intelligence via agentic retrieval-augmented language models</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/computers15040203</t>
+          <t>https://doi.org/10.3389/fnut.2026.1815038</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5612,7 +5616,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BIO-134</t>
+          <t>BIO-131</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -5623,12 +5627,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>An Adaptive Multi-Agent LLM-Based Clinical Decision Support System Integrating Biomedical RAG and Web Intelligence</t>
+          <t>MEGA-RAG: a retrieval-augmented generation framework with multi-evidence guided answer refinement for mitigating hallucinations of LLMs in public health</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/access.2025.3613340</t>
+          <t>https://doi.org/10.3389/fpubh.2025.1635381</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5650,7 +5654,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>BIO-135</t>
+          <t>BIO-132</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -5661,12 +5665,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>A self-correcting Agentic Graph RAG for clinical decision support in hepatology</t>
+          <t>Use of Retrieval-Augmented Large Language Model for COVID-19 Fact-Checking: Development and Usability Study</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/fmed.2025.1716327</t>
+          <t>https://doi.org/10.2196/66098</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5688,7 +5692,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>BIO-136</t>
+          <t>BIO-133</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
@@ -5699,12 +5703,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>A novel context-aware retrieval framework for biomedical knowledge integration with large language models</t>
+          <t>GraphRAG-Vet: A Knowledge Graph-Augmented Large Language Model for Precision Bovine Disease Diagnosis</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.inffus.2025.103902</t>
+          <t>https://doi.org/10.3390/computers15040203</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5726,7 +5730,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>BIO-137</t>
+          <t>BIO-134</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -5737,12 +5741,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Using large language models to assist antimicrobial resistance policy development: Integrating the environment into health protection planning</t>
+          <t>An Adaptive Multi-Agent LLM-Based Clinical Decision Support System Integrating Biomedical RAG and Web Intelligence</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1021/acs.est.4c07842</t>
+          <t>https://doi.org/10.1109/access.2025.3613340</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5764,7 +5768,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BIO-139</t>
+          <t>BIO-135</t>
         </is>
       </c>
       <c r="B123" t="inlineStr"/>
@@ -5775,25 +5779,177 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
+          <t>A self-correcting Agentic Graph RAG for clinical decision support in hepatology</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fmed.2025.1716327</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>prefiltro</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>BIO-136</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Tema a revisar</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>A novel context-aware retrieval framework for biomedical knowledge integration with large language models</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.inffus.2025.103902</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>prefiltro</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>BIO-137</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Tema a revisar</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Using large language models to assist antimicrobial resistance policy development: Integrating the environment into health protection planning</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.est.4c07842</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>prefiltro</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>BIO-138</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Tema a revisar</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>VAIV bio-discovery service using transformer model and retrieval augmented generation</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12859-024-05903-6</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>prefiltro</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>BIO-139</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Tema a revisar</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
           <t>Retrieval augmented generation system for mental health information</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E127" t="inlineStr">
         <is>
           <t>https://doi.org/10.3233/shti250929</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
+      <c r="F127" t="inlineStr">
         <is>
           <t>Excluido a mano: paper de LLM/salud mental en bioseguridad (para revisar por Investigación)</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr">
+      <c r="G127" t="inlineStr">
         <is>
           <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr">
+      <c r="H127" t="inlineStr">
         <is>
           <t>prefiltro</t>
         </is>

</xml_diff>

<commit_message>
Corpus: Excel de fuentes E4 y D3 indexado tambien en bioseguridad_md (reemplaza a F1)
</commit_message>
<xml_diff>
--- a/corpus/md/para_investigacion.xlsx
+++ b/corpus/md/para_investigacion.xlsx
@@ -415,13 +415,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Para revisar por Investigación (generado el 2026-10-15 03:30)</t>
+          <t>Para revisar por Investigación (generado el 2026-10-28 01:09)</t>
         </is>
       </c>
     </row>
@@ -489,10 +489,10 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -526,73 +526,73 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
       </c>
       <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E6" t="n">
         <v>3</v>
       </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Sin ruta</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
         <v>1</v>
-      </c>
-      <c r="F8" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sin ruta</t>
+          <t>Sin texto</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -602,101 +602,79 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sin texto</t>
+          <t>Solo resumen</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>0</v>
       </c>
       <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
         <v>1</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Solo resumen</t>
+          <t>Tema a revisar</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tema a revisar</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>22</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F12" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>22</v>
-      </c>
-      <c r="C13" t="n">
-        <v>47</v>
-      </c>
-      <c r="D13" t="n">
-        <v>32</v>
-      </c>
-      <c r="E13" t="n">
-        <v>25</v>
-      </c>
-      <c r="F13" t="n">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -710,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2270,7 +2248,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2285,12 +2263,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Case Definition: Avian Influenza (AI) in Poultry (Notifiable)</t>
+          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://www.aphis.usda.gov/sites/default/files/avian-influenza-case-definition.pdf</t>
+          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2312,12 +2290,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2327,17 +2305,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
+          <t>Genetic data and meteorological conditions suggesting windborne transmission of H5N1 high-pathogenicity avian influenza between commercial poultry outbreaks</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
+          <t>https://www.biorxiv.org/content/10.1101/2025.02.12.637829</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>d) PDF directo: sin respuesta en 10 s</t>
+          <t>c) Web: www.biorxiv.org no disponible (HTTP 429) | c) Web: www.biorxiv.org no disponible (HTTP 429)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3446,7 +3424,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>E1</t>
+          <t>BIO-001</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3456,39 +3434,39 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Ley 18.755 – Establece normas sobre el Servicio Agrícola y Ganadero (Ley Orgánica del SAG)</t>
+          <t>Determinants of biosecurity practices in French duck farms after a H5N8 Highly Pathogenic Avian Influenza epidemic: The effect of farmer knowledge, attitudes and personality traits</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://www.bcn.cl/leychile/navegar?idNorma=30135</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13462</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>título 46/100 y 31 palabras</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>LeyChile necesita JavaScript y reCAPTCHA: bajar a mano el PDF de la norma.</t>
+          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>BIO-006</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3498,39 +3476,39 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Brote Influenza aviar 2026. Antecedentes generales y situación nacional (Asesoría Técnica Parlamentaria)</t>
+          <t>Factors influencing chicken farmers' decisions to implement prevention and control measures to reduce avian influenza virus spread under endemic conditions</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://www.bcn.cl/asesoriasparlamentarias/detalle_documento.html?id=85550</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13757</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>título 42/100 y 17 palabras</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>LeyChile necesita JavaScript y reCAPTCHA: bajar a mano el PDF de la norma.</t>
+          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>BIO-018</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3540,123 +3518,123 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Resolución Exenta N° 4.869 – Medidas sanitarias y obligaciones para terceros en contexto de enfermedades declaradas bajo control oficial</t>
+          <t>A systematic approach to illuminate a new hot spot of avian influenza virus circulation in South Vietnam, 2016–2017</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://www.bcn.cl/leychile/navegar?idNorma=1224888</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14380</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>título 41/100 y 31 palabras</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>LeyChile necesita JavaScript y reCAPTCHA: bajar a mano el PDF de la norma.</t>
+          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>A13</t>
+          <t>BIO-073</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Effect of temperature-humidity index on live performance in broiler chickens grown from 49 to 63 days of age</t>
+          <t>Veterinarians' knowledge and experience of avian influenza and perspectives on control measures in the UK</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://works.bepress.com/hongwei_xin/134</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/vetr.3713</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>título 41/100 y 60 palabras</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>La URL no lleva al documento: poner el link directo o el PDF.</t>
+          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>A15</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Página equivocada</t>
+          <t>Rechazado por la editorial</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Descripcion y usos de la Red de Agrometeorologia INIA (Boletin INIA N 415)</t>
+          <t>Modifications to the hemagglutinin cleavage site control the virulence of a neurotropic H1N1 influenza virus</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://sitios.inia.cl/agrometeorologia/boletin-415/</t>
+          <t>https://journals.asm.org/doi/10.1128/jvi.00797-10</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>título 79/100 y 121 palabras</t>
+          <t>c) Web: journals.asm.org rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>La URL no lleva al documento: poner el link directo o el PDF.</t>
+          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BIO-001</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3671,17 +3649,17 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Determinants of biosecurity practices in French duck farms after a H5N8 Highly Pathogenic Avian Influenza epidemic: The effect of farmer knowledge, attitudes and personality traits</t>
+          <t>Abiotic factors affecting the persistence of avian influenza virus in surface waters of waterfowl habitats</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13462</t>
+          <t>https://aem.asm.org/content/aem/80/9/2910.full.pdf</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>aem.asm.org rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3698,12 +3676,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BIO-006</t>
+          <t>A12</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3713,17 +3691,17 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Factors influencing chicken farmers' decisions to implement prevention and control measures to reduce avian influenza virus spread under endemic conditions</t>
+          <t>Heat stress impairs performance and induces intestinal inflammation in broiler chickens infected with Salmonella Enteritidis</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.13757</t>
+          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2012.709315?needAccess=true&amp;role=button</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>www.tandfonline.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3740,12 +3718,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BIO-018</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3755,17 +3733,17 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>A systematic approach to illuminate a new hot spot of avian influenza virus circulation in South Vietnam, 2016–2017</t>
+          <t>Inactivation of the infectivity of two highly pathogenic avian influenza viruses and a virulent Newcastle disease virus by ultraviolet radiation</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14380</t>
+          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2013.853867?needAccess=true&amp;role=button</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>www.tandfonline.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3782,12 +3760,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BIO-073</t>
+          <t>CLI-005</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3797,17 +3775,17 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Veterinarians' knowledge and experience of avian influenza and perspectives on control measures in the UK</t>
+          <t>Determinants of highly pathogenic avian influenza spread during bird migration</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/vetr.3713</t>
+          <t>https://doi.org/10.1098/rsos.260182</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: royalsocietypublishing.org rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3817,19 +3795,19 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>C19</t>
+          <t>CLI-023</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3839,17 +3817,17 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Modifications to the hemagglutinin cleavage site control the virulence of a neurotropic H1N1 influenza virus</t>
+          <t>A threat from both sides: Multiple introductions of genetically distinct H5 HPAI viruses into Canada via both East Asia-Australasia/Pacific and Atlantic flyways.</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://journals.asm.org/doi/10.1128/jvi.00797-10</t>
+          <t>https://doi.org/10.1093/ve/veac077</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>c) Web: journals.asm.org rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: academic.oup.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3866,12 +3844,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>CLI-043</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3881,17 +3859,17 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Abiotic factors affecting the persistence of avian influenza virus in surface waters of waterfowl habitats</t>
+          <t>Global dissemination of influenza A virus is driven by wild bird migration through arctic and subarctic zones.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://aem.asm.org/content/aem/80/9/2910.full.pdf</t>
+          <t>https://www.authorea.com/doi/pdf/10.22541/au.164372348.88612449</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>aem.asm.org rechaza el acceso (HTTP 403)</t>
+          <t>www.authorea.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3908,7 +3886,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>A12</t>
+          <t>CLI-059</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3923,17 +3901,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Heat stress impairs performance and induces intestinal inflammation in broiler chickens infected with Salmonella Enteritidis</t>
+          <t>Waterfowl show spatiotemporal trends in influenza A H5 and H7 infections but limited taxonomic variation.</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2012.709315?needAccess=true&amp;role=button</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/eap.2906</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>www.tandfonline.com rechaza el acceso (HTTP 403)</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3950,7 +3928,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>CLI-061</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3965,17 +3943,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Inactivation of the infectivity of two highly pathogenic avian influenza viruses and a virulent Newcastle disease virus by ultraviolet radiation</t>
+          <t>Seasonality of influenza and coseasonality with avian influenza in Bangladesh, 2010-19: a retrospective, time-series analysis.</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://www.tandfonline.com/doi/pdf/10.1080/03079457.2013.853867?needAccess=true&amp;role=button</t>
+          <t>http://www.thelancet.com/article/S2214109X22002121/pdf</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>www.tandfonline.com rechaza el acceso (HTTP 403)</t>
+          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3992,7 +3970,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CLI-005</t>
+          <t>CLI-068</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4007,17 +3985,17 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Determinants of highly pathogenic avian influenza spread during bird migration</t>
+          <t>Improved method for avian influenza virus isolation from environmental water samples.</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1098/rsos.260182</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14639</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>c) Web: royalsocietypublishing.org rechaza el acceso (HTTP 403)</t>
+          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -4027,14 +4005,14 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CLI-023</t>
+          <t>CLI-090</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4049,17 +4027,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>A threat from both sides: Multiple introductions of genetically distinct H5 HPAI viruses into Canada via both East Asia-Australasia/Pacific and Atlantic flyways.</t>
+          <t>Spatiotemporal patterns of low and highly pathogenic avian influenza virus prevalence in murres in Canada from 2007 to 2022—a case study for wildlife viral monitoring</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1093/ve/veac077</t>
+          <t>https://doi.org/10.1139/facets-2023-0185</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>c) Web: academic.oup.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: www.facetsjournal.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4076,7 +4054,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CLI-043</t>
+          <t>CLI-119</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4091,17 +4069,17 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Global dissemination of influenza A virus is driven by wild bird migration through arctic and subarctic zones.</t>
+          <t>Cost of migration increased during an outbreak of highly pathogenic avian influenza virus</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://www.authorea.com/doi/pdf/10.22541/au.164372348.88612449</t>
+          <t>https://doi.org/10.1002/jav.03616</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>www.authorea.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: nsojournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4111,14 +4089,14 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CLI-059</t>
+          <t>CLI-130</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4133,17 +4111,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Waterfowl show spatiotemporal trends in influenza A H5 and H7 infections but limited taxonomic variation.</t>
+          <t>Integrating wild bird and environmental samples can strengthen avian influenza surveillance</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1002/eap.2906</t>
+          <t>https://doi.org/10.1111/1365-2664.70584</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>c) Web: besjournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4153,19 +4131,19 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CLI-061</t>
+          <t>D-PM110</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4175,17 +4153,17 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Seasonality of influenza and coseasonality with avian influenza in Bangladesh, 2010-19: a retrospective, time-series analysis.</t>
+          <t>Surveillance of avian influenza viruses in Hebei Province of China from 2021 to 2023: Identification of a novel reassortant H3N3.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>http://www.thelancet.com/article/S2214109X22002121/pdf</t>
+          <t>https://www.journalofinfection.com/article/S0163-4453(24)00174-9/pdf</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
+          <t>www.journalofinfection.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4202,12 +4180,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CLI-068</t>
+          <t>D-PM139</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4217,17 +4195,17 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Improved method for avian influenza virus isolation from environmental water samples.</t>
+          <t>Wastewater monitoring of human and avian influenza A viruses in Northern Ireland: a genomic surveillance study.</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/tbed.14639</t>
+          <t>http://www.thelancet.com/article/S2666524724001757/pdf</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4244,12 +4222,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CLI-090</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4259,17 +4237,17 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Spatiotemporal patterns of low and highly pathogenic avian influenza virus prevalence in murres in Canada from 2007 to 2022—a case study for wildlife viral monitoring</t>
+          <t>The MIQE Guidelines: Minimum Information for Publication of Quantitative Real-Time PCR Experiments</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1139/facets-2023-0185</t>
+          <t>http://clinchem.aaccjnls.org/content/clinchem/55/4/611.full.pdf</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>c) Web: www.facetsjournal.com rechaza el acceso (HTTP 403)</t>
+          <t>academic.oup.com rechaza el acceso (HTTP 403)</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4279,224 +4257,224 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CLI-119</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Cost of migration increased during an outbreak of highly pathogenic avian influenza virus</t>
+          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1002/jav.03616</t>
+          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>c) Web: nsojournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>título 69/100 (&lt; 80) y 1083 palabras</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
+          <t>Abrir el .md y confirmar que es el documento correcto.</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CLI-130</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>climatico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Integrating wild bird and environmental samples can strengthen avian influenza surveillance</t>
+          <t>Codigo Sanitario para los Animales Terrestres, Capitulo 1.1: Notificacion de enfermedades y presentacion de datos epidemiologicos (articulo 1.1.3)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1111/1365-2664.70584</t>
+          <t>https://www.woah.org/fileadmin/Home/eng/Health_standards/tahc/2023/chapitre_notification.pdf</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>c) Web: besjournals.onlinelibrary.wiley.com rechaza el acceso (HTTP 403)</t>
+          <t>título 58/100 (&lt; 80) y 1108 palabras</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
+          <t>Abrir el .md y confirmar que es el documento correcto.</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>prefiltro</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>D-PM110</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Surveillance of avian influenza viruses in Hebei Province of China from 2021 to 2023: Identification of a novel reassortant H3N3.</t>
+          <t>SAG logra en tiempo record la reapertura de los principales mercados de productos avicolas tras foco de influenza aviar (comunicado)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://www.journalofinfection.com/article/S0163-4453(24)00174-9/pdf</t>
+          <t>https://www.sag.gob.cl/noticias/sag-logra-en-tiempo-record-la-reapertura-de-los-principales-mercados-de-productos-avicolas-tras-foco-de-influenza-aviar</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>www.journalofinfection.com rechaza el acceso (HTTP 403)</t>
+          <t>título 53/100 (&lt; 80) y 431 palabras</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
+          <t>Abrir el .md y confirmar que es el documento correcto.</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>D-PM139</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Wastewater monitoring of human and avian influenza A viruses in Northern Ireland: a genomic surveillance study.</t>
+          <t>Chile se autodeclara pais libre de influenza aviar altamente patogena en aves de corral (comunicado)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>http://www.thelancet.com/article/S2666524724001757/pdf</t>
+          <t>https://www.sag.gob.cl/noticias/chile-se-autodeclara-pais-libre-de-influenza-aviar-altamente-patogena-en-aves-de-corral</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>www.thelancet.com rechaza el acceso (HTTP 403)</t>
+          <t>título 70/100 (&lt; 80) y 717 palabras</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
+          <t>Abrir el .md y confirmar que es el documento correcto.</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>bioseguridad</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Rechazado por la editorial</t>
+          <t>Revisar título</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>The MIQE Guidelines: Minimum Information for Publication of Quantitative Real-Time PCR Experiments</t>
+          <t>SAG – Pecuaria (ámbito de acción)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>http://clinchem.aaccjnls.org/content/clinchem/55/4/611.full.pdf</t>
+          <t>https://www.sag.gob.cl/ambitos-de-accion/pecuaria</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>academic.oup.com rechaza el acceso (HTTP 403)</t>
+          <t>título 59/100 (&lt; 80) y 487 palabras</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>El sitio bloquea bots: bajar el PDF a mano.</t>
+          <t>Abrir el .md y confirmar que es el documento correcto.</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>validación</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>E19</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4511,17 +4489,17 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Depopulation and disposal - HPAI response (ficha informativa)</t>
+          <t>SAG – Resolución Exenta N° 7.050: aprueba Instructivo Técnico de Bioseguridad de las Personas (influenza aviar), versión 3</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://www.aphis.usda.gov/sites/default/files/hpai-depopulation-disposal.pdf</t>
+          <t>https://www.sag.gob.cl/content/aprueba-instructivo-tecnico-de-bioseguridad-de-las-personas-en-una-emergencia-zoosanitaria-con-riesgo-de-zoonosis-influenza-aviar-ia-version-3-y-dejese-sin-efecto-la-resolucion-exenta-ndeg-39962026</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>título 69/100 (&lt; 80) y 1083 palabras</t>
+          <t>título 79/100 (&lt; 80) y 339 palabras</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4538,7 +4516,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>C22</t>
+          <t>E21</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4553,17 +4531,17 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Codigo Sanitario para los Animales Terrestres, Capitulo 1.1: Notificacion de enfermedades y presentacion de datos epidemiologicos (articulo 1.1.3)</t>
+          <t>FAO – EMPRES-i (página 'Acerca de' del sitio data.apps.fao.org)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://www.woah.org/fileadmin/Home/eng/Health_standards/tahc/2023/chapitre_notification.pdf</t>
+          <t>https://data.apps.fao.org/static/sites/empres-i/about.html</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>título 58/100 (&lt; 80) y 1108 palabras</t>
+          <t>título 56/100 (&lt; 80) y 239 palabras</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4580,7 +4558,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>C32</t>
+          <t>E23</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4595,17 +4573,17 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>SAG logra en tiempo record la reapertura de los principales mercados de productos avicolas tras foco de influenza aviar (comunicado)</t>
+          <t>FAO – Preguntas frecuentes sobre EMA-i+ y EMPRES-i+</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/noticias/sag-logra-en-tiempo-record-la-reapertura-de-los-principales-mercados-de-productos-avicolas-tras-foco-de-influenza-aviar</t>
+          <t>https://www.fao.org/animal-health/resources/tools/faq-ema-i-empres-i/en</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>título 53/100 (&lt; 80) y 431 palabras</t>
+          <t>título 64/100 (&lt; 80) y 504 palabras</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4622,7 +4600,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>C33</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4637,17 +4615,17 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Chile se autodeclara pais libre de influenza aviar altamente patogena en aves de corral (comunicado)</t>
+          <t>FAO – EMPRES-i (proyecto en AgroInformática)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/noticias/chile-se-autodeclara-pais-libre-de-influenza-aviar-altamente-patogena-en-aves-de-corral</t>
+          <t>https://www.fao.org/agroinformatics/projects/projects-detail/empres-i/</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>título 70/100 (&lt; 80) y 717 palabras</t>
+          <t>título 67/100 (&lt; 80) y 242 palabras</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4664,12 +4642,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>diagnostico</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4679,17 +4657,13 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>SAG – Pecuaria (ámbito de acción)</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>https://www.sag.gob.cl/ambitos-de-accion/pecuaria</t>
-        </is>
-      </c>
+          <t>IDEXX PRRS X3 Ab Test - pagina de producto</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>título 59/100 (&lt; 80) y 487 palabras</t>
+          <t>título 64/100 (&lt; 80) y 173 palabras</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4706,7 +4680,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>E19</t>
+          <t>BIO-118</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4716,39 +4690,39 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Sin ruta</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>SAG – Resolución Exenta N° 7.050: aprueba Instructivo Técnico de Bioseguridad de las Personas (influenza aviar), versión 3</t>
+          <t>Building trustworthy generative artificial intelligence for diabetes care and limb preservation: a medical knowledge extraction case</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://www.sag.gob.cl/content/aprueba-instructivo-tecnico-de-bioseguridad-de-las-personas-en-una-emergencia-zoosanitaria-con-riesgo-de-zoonosis-influenza-aviar-ia-version-3-y-dejese-sin-efecto-la-resolucion-exenta-ndeg-39962026</t>
+          <t>https://doi.org/10.1177/19322968241253568</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>título 79/100 (&lt; 80) y 339 palabras</t>
+          <t>solo hay la web de PMC, que no se usa (CAPTCHA); falta texto en Europe PMC</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Abrir el .md y confirmar que es el documento correcto.</t>
+          <t>Buscar el link directo al documento o el PDF.</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>E21</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4758,149 +4732,153 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Sin texto</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>FAO – EMPRES-i (página 'Acerca de' del sitio data.apps.fao.org)</t>
+          <t>Protocolo de vigilancia ocupacional por exposición a influenza aviar, versión 2</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://data.apps.fao.org/static/sites/empres-i/about.html</t>
+          <t>https://www.achs.cl/docs/librariesprovider2/empresa/20-gripe-aviar/legales/protocolo-de-vigilancia-ocupacional-por-exposicion-a-influenza-aviar-version-2.pdf</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>título 56/100 (&lt; 80) y 239 palabras</t>
+          <t>no se pudo sacar texto</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Abrir el .md y confirmar que es el documento correcto.</t>
+          <t>No se pudo sacar texto: revisar el archivo.</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>E23</t>
+          <t>CLI-081</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Sin texto</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>FAO – Preguntas frecuentes sobre EMA-i+ y EMPRES-i+</t>
+          <t>A SYSTEMATIC REVIEW AND NARRATIVE SYNTHESIS OF THE USE OF ENVIRONMENTAL SAMPLES FOR THE SURVEILLANCE OF AVIAN INFLUENZA VIRUSES IN WILD WATERBIRDS.</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://www.fao.org/animal-health/resources/tools/faq-ema-i-empres-i/en</t>
+          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-57/issue-1/JWD-D-20-00082/A-SYSTEMATIC-REVIEW-AND-NARRATIVE-SYNTHESIS-OF-THE-USE-OF/10.7589/JWD-D-20-00082.pdf</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>título 64/100 (&lt; 80) y 504 palabras</t>
+          <t>se esperaba un PDF y llegó una página web</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Abrir el .md y confirmar que es el documento correcto.</t>
+          <t>No se pudo sacar texto: revisar el archivo.</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>E24</t>
+          <t>CLI-105</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>bioseguridad</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Sin texto</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>FAO – EMPRES-i (proyecto en AgroInformática)</t>
+          <t>Pathogen Surveillance in Swallows (family Hirundinidae): Investigation into Role as Avian Influenza Vector in Eastern Canada Agricultural Landscapes.</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://www.fao.org/agroinformatics/projects/projects-detail/empres-i/</t>
+          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-60/issue-3/JWD-D-23-00167/Pathogen-Surveillance-in-Swallows-Family-Hirundinidae--Investigation-into-Role/10.7589/JWD-D-23-00167.pdf</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>título 67/100 (&lt; 80) y 242 palabras</t>
+          <t>se esperaba un PDF y llegó una página web</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Abrir el .md y confirmar que es el documento correcto.</t>
+          <t>No se pudo sacar texto: revisar el archivo.</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>descarga</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>diagnostico</t>
+          <t>climatico</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Revisar título</t>
+          <t>Solo resumen</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>IDEXX PRRS X3 Ab Test - pagina de producto</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr"/>
+          <t>Genetic data and meteorological conditions: unravelling the windborne transmission of H5N1 high-pathogenicity avian influenza between commercial poultry outbreaks</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://www.biorxiv.org/content/10.1101/2025.02.12.637829</t>
+        </is>
+      </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>título 64/100 (&lt; 80) y 173 palabras</t>
+          <t>Abstract sin Methods/Results/Discussion y 261 palabras</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Abrir el .md y confirmar que es el documento correcto.</t>
+          <t>Solo llegó el resumen: conseguir el texto completo.</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4912,37 +4890,33 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BIO-118</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>bioseguridad</t>
-        </is>
-      </c>
+          <t>BIO-117</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Sin ruta</t>
+          <t>Tema a revisar</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Building trustworthy generative artificial intelligence for diabetes care and limb preservation: a medical knowledge extraction case</t>
+          <t>Answering real-world clinical questions using large language model, retrieval-augmented generation, and agentic systems</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/19322968241253568</t>
+          <t>https://doi.org/10.1177/20552076251348850</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>solo hay la web de PMC, que no se usa (CAPTCHA); falta texto en Europe PMC</t>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Buscar el link directo al documento o el PDF.</t>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4954,175 +4928,159 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>bioseguridad</t>
-        </is>
-      </c>
+          <t>BIO-119</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Sin texto</t>
+          <t>Tema a revisar</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>PROTOCOLO DE VIGILANCIA OCUPACIONAL POR EXPOSICIÓN A INFLUENZA AVIAR Versión Nº2</t>
+          <t>From RAGs to riches: utilizing large language models to write documents for clinical trials</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://www.achs.cl/docs/librariesprovider2/empresa/20-gripe-aviar/legales/protocolo-de-vigilancia-ocupacional-por-exposicion-a-influenza-aviar-version-2.pdf</t>
+          <t>https://doi.org/10.1177/17407745251320806</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>no se pudo sacar texto</t>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>No se pudo sacar texto: revisar el archivo.</t>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CLI-081</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>climatico</t>
-        </is>
-      </c>
+          <t>BIO-120</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Sin texto</t>
+          <t>Tema a revisar</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>A SYSTEMATIC REVIEW AND NARRATIVE SYNTHESIS OF THE USE OF ENVIRONMENTAL SAMPLES FOR THE SURVEILLANCE OF AVIAN INFLUENZA VIRUSES IN WILD WATERBIRDS.</t>
+          <t>Evaluating adherence to Canadian radiology guidelines for incidental hepatobiliary findings using RAG-enabled LLMs</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-57/issue-1/JWD-D-20-00082/A-SYSTEMATIC-REVIEW-AND-NARRATIVE-SYNTHESIS-OF-THE-USE-OF/10.7589/JWD-D-20-00082.pdf</t>
+          <t>https://doi.org/10.1177/08465371251323124</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>se esperaba un PDF y llegó una página web</t>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>No se pudo sacar texto: revisar el archivo.</t>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CLI-105</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>climatico</t>
-        </is>
-      </c>
+          <t>BIO-121</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Sin texto</t>
+          <t>Tema a revisar</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Pathogen Surveillance in Swallows (family Hirundinidae): Investigation into Role as Avian Influenza Vector in Eastern Canada Agricultural Landscapes.</t>
+          <t>LLM-augmented multi-agent cooperative framework for medical case retrieval in cardiology</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://bioone.org/journals/journal-of-wildlife-diseases/volume-60/issue-3/JWD-D-23-00167/Pathogen-Surveillance-in-Swallows-Family-Hirundinidae--Investigation-into-Role/10.7589/JWD-D-23-00167.pdf</t>
+          <t>https://doi.org/10.1007/s44443-025-00311-z</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>se esperaba un PDF y llegó una página web</t>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>No se pudo sacar texto: revisar el archivo.</t>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>descarga</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>A3</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>climatico</t>
-        </is>
-      </c>
+          <t>BIO-122</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Solo resumen</t>
+          <t>Tema a revisar</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Genetic data and meteorological conditions: unravelling the windborne transmission of H5N1 high-pathogenicity avian influenza between commercial poultry outbreaks</t>
+          <t>Performance of latest AI models, RAG, and MCP on lung cancer-related questions</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://www.biorxiv.org/content/10.1101/2025.02.12.637829</t>
+          <t>https://doi.org/10.1177/20552076261427503</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Abstract sin Methods/Results/Discussion y 261 palabras</t>
+          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Solo llegó el resumen: conseguir el texto completo.</t>
+          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>validación</t>
+          <t>prefiltro</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BIO-117</t>
+          <t>BIO-123</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
@@ -5133,12 +5091,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Answering real-world clinical questions using large language model, retrieval-augmented generation, and agentic systems</t>
+          <t>BIOGEN: evidence-grounded multi-agent reasoning framework for transcriptomic interpretation in antimicrobial resistance</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076251348850</t>
+          <t>https://doi.org/10.3389/fbinf.2026.1846404</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -5160,7 +5118,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>BIO-119</t>
+          <t>BIO-124</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
@@ -5171,12 +5129,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>From RAGs to riches: utilizing large language models to write documents for clinical trials</t>
+          <t>A Chatbot for the Management of Bipolar Disorder: Using Retrieval-Augmented Generation With an Open-Weight Large Language Model to Answer Clinical Questions Based on the CANMAT and ISBD 2018 Guidelines for Bipolar Disorder: Un dialogueur pour la prise en charge du trouble bipolaire : utiliser la génération augmentée par récupération avec un grand modèle de langage (GML) à poids ouverts pour répondre aux questions cliniques fondées sur les lignes directrices de 2018 de CANMAT et de l'ISBD relatives au trouble bipolaire</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/17407745251320806</t>
+          <t>https://doi.org/10.1177/07067437261457232</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -5198,7 +5156,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>BIO-120</t>
+          <t>BIO-125</t>
         </is>
       </c>
       <c r="B108" t="inlineStr"/>
@@ -5209,12 +5167,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Evaluating adherence to Canadian radiology guidelines for incidental hepatobiliary findings using RAG-enabled LLMs</t>
+          <t>Development of a cancer information chatbot model: Retrieval-augmented generation with data from the national center for cancer knowledge and information</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/08465371251323124</t>
+          <t>https://doi.org/10.1177/20552076261450314</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -5236,7 +5194,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BIO-121</t>
+          <t>BIO-126</t>
         </is>
       </c>
       <c r="B109" t="inlineStr"/>
@@ -5247,12 +5205,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>LLM-augmented multi-agent cooperative framework for medical case retrieval in cardiology</t>
+          <t>Improved accuracy and efficiency of guideline-based orthopedic disability assessment with a retrieval-augmented AI assistant (NotebookLM) in anonymized cases</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1007/s44443-025-00311-z</t>
+          <t>https://doi.org/10.1177/20552076261473719</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -5274,7 +5232,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BIO-122</t>
+          <t>BIO-127</t>
         </is>
       </c>
       <c r="B110" t="inlineStr"/>
@@ -5285,12 +5243,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Performance of latest AI models, RAG, and MCP on lung cancer-related questions</t>
+          <t>Performance and usability of retrieval-augmented large language models for stroke patient and caregiver support</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261427503</t>
+          <t>https://doi.org/10.1177/20552076261464997</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5312,7 +5270,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>BIO-123</t>
+          <t>BIO-128</t>
         </is>
       </c>
       <c r="B111" t="inlineStr"/>
@@ -5323,12 +5281,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>BIOGEN: evidence-grounded multi-agent reasoning framework for transcriptomic interpretation in antimicrobial resistance</t>
+          <t>Design and multidimensional expert evaluation of a national health information portal-integrated generative AI chatbot for health literacy and awareness</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/fbinf.2026.1846404</t>
+          <t>https://doi.org/10.1177/20552076261481326</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -5350,7 +5308,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BIO-124</t>
+          <t>BIO-129</t>
         </is>
       </c>
       <c r="B112" t="inlineStr"/>
@@ -5361,12 +5319,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>A Chatbot for the Management of Bipolar Disorder: Using Retrieval-Augmented Generation With an Open-Weight Large Language Model to Answer Clinical Questions Based on the CANMAT and ISBD 2018 Guidelines for Bipolar Disorder: Un dialogueur pour la prise en charge du trouble bipolaire : utiliser la génération augmentée par récupération avec un grand modèle de langage (GML) à poids ouverts pour répondre aux questions cliniques fondées sur les lignes directrices de 2018 de CANMAT et de l'ISBD relatives au trouble bipolaire</t>
+          <t>Dynamic alignment of large language models for evidence-grounded heart failure decision support</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/07067437261457232</t>
+          <t>https://doi.org/10.1177/20552076261487568</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5388,7 +5346,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BIO-125</t>
+          <t>BIO-130</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
@@ -5399,12 +5357,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Development of a cancer information chatbot model: Retrieval-augmented generation with data from the national center for cancer knowledge and information</t>
+          <t>Toward an integrated animal–human nutrition intelligence via agentic retrieval-augmented language models</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261450314</t>
+          <t>https://doi.org/10.3389/fnut.2026.1815038</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5426,7 +5384,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>BIO-126</t>
+          <t>BIO-131</t>
         </is>
       </c>
       <c r="B114" t="inlineStr"/>
@@ -5437,12 +5395,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Improved accuracy and efficiency of guideline-based orthopedic disability assessment with a retrieval-augmented AI assistant (NotebookLM) in anonymized cases</t>
+          <t>MEGA-RAG: a retrieval-augmented generation framework with multi-evidence guided answer refinement for mitigating hallucinations of LLMs in public health</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261473719</t>
+          <t>https://doi.org/10.3389/fpubh.2025.1635381</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5464,7 +5422,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>BIO-127</t>
+          <t>BIO-132</t>
         </is>
       </c>
       <c r="B115" t="inlineStr"/>
@@ -5475,12 +5433,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Performance and usability of retrieval-augmented large language models for stroke patient and caregiver support</t>
+          <t>Use of Retrieval-Augmented Large Language Model for COVID-19 Fact-Checking: Development and Usability Study</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261464997</t>
+          <t>https://doi.org/10.2196/66098</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5502,7 +5460,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>BIO-128</t>
+          <t>BIO-133</t>
         </is>
       </c>
       <c r="B116" t="inlineStr"/>
@@ -5513,12 +5471,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Design and multidimensional expert evaluation of a national health information portal-integrated generative AI chatbot for health literacy and awareness</t>
+          <t>GraphRAG-Vet: A Knowledge Graph-Augmented Large Language Model for Precision Bovine Disease Diagnosis</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261481326</t>
+          <t>https://doi.org/10.3390/computers15040203</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5540,7 +5498,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>BIO-129</t>
+          <t>BIO-134</t>
         </is>
       </c>
       <c r="B117" t="inlineStr"/>
@@ -5551,12 +5509,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Dynamic alignment of large language models for evidence-grounded heart failure decision support</t>
+          <t>An Adaptive Multi-Agent LLM-Based Clinical Decision Support System Integrating Biomedical RAG and Web Intelligence</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1177/20552076261487568</t>
+          <t>https://doi.org/10.1109/access.2025.3613340</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5578,7 +5536,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>BIO-130</t>
+          <t>BIO-135</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
@@ -5589,12 +5547,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Toward an integrated animal–human nutrition intelligence via agentic retrieval-augmented language models</t>
+          <t>A self-correcting Agentic Graph RAG for clinical decision support in hepatology</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/fnut.2026.1815038</t>
+          <t>https://doi.org/10.3389/fmed.2025.1716327</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5616,7 +5574,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BIO-131</t>
+          <t>BIO-136</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
@@ -5627,12 +5585,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>MEGA-RAG: a retrieval-augmented generation framework with multi-evidence guided answer refinement for mitigating hallucinations of LLMs in public health</t>
+          <t>A novel context-aware retrieval framework for biomedical knowledge integration with large language models</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3389/fpubh.2025.1635381</t>
+          <t>https://doi.org/10.1016/j.inffus.2025.103902</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5654,7 +5612,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>BIO-132</t>
+          <t>BIO-137</t>
         </is>
       </c>
       <c r="B120" t="inlineStr"/>
@@ -5665,12 +5623,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Use of Retrieval-Augmented Large Language Model for COVID-19 Fact-Checking: Development and Usability Study</t>
+          <t>Using large language models to assist antimicrobial resistance policy development: Integrating the environment into health protection planning</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://doi.org/10.2196/66098</t>
+          <t>https://doi.org/10.1021/acs.est.4c07842</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5692,7 +5650,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>BIO-133</t>
+          <t>BIO-138</t>
         </is>
       </c>
       <c r="B121" t="inlineStr"/>
@@ -5703,12 +5661,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>GraphRAG-Vet: A Knowledge Graph-Augmented Large Language Model for Precision Bovine Disease Diagnosis</t>
+          <t>VAIV bio-discovery service using transformer model and retrieval augmented generation</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/computers15040203</t>
+          <t>https://doi.org/10.1186/s12859-024-05903-6</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5730,7 +5688,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>BIO-134</t>
+          <t>BIO-139</t>
         </is>
       </c>
       <c r="B122" t="inlineStr"/>
@@ -5741,17 +5699,17 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>An Adaptive Multi-Agent LLM-Based Clinical Decision Support System Integrating Biomedical RAG and Web Intelligence</t>
+          <t>Retrieval augmented generation system for mental health information</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1109/access.2025.3613340</t>
+          <t>https://doi.org/10.3233/shti250929</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
+          <t>Excluido a mano: paper de LLM/salud mental en bioseguridad (para revisar por Investigación)</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -5760,196 +5718,6 @@
         </is>
       </c>
       <c r="H122" t="inlineStr">
-        <is>
-          <t>prefiltro</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>BIO-135</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Tema a revisar</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>A self-correcting Agentic Graph RAG for clinical decision support in hepatology</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3389/fmed.2025.1716327</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>prefiltro</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>BIO-136</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Tema a revisar</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>A novel context-aware retrieval framework for biomedical knowledge integration with large language models</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1016/j.inffus.2025.103902</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr">
-        <is>
-          <t>prefiltro</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>BIO-137</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Tema a revisar</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>Using large language models to assist antimicrobial resistance policy development: Integrating the environment into health protection planning</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1021/acs.est.4c07842</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr">
-        <is>
-          <t>prefiltro</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>BIO-138</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Tema a revisar</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>VAIV bio-discovery service using transformer model and retrieval augmented generation</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1186/s12859-024-05903-6</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Excluido a mano: paper de LLM/RAG en bioseguridad, no es base veterinaria (para revisar por Investigación)</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>prefiltro</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>BIO-139</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Tema a revisar</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Retrieval augmented generation system for mental health information</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.3233/shti250929</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>Excluido a mano: paper de LLM/salud mental en bioseguridad (para revisar por Investigación)</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>¿Es base veterinaria? Si no, sacarlo del Excel.</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr">
         <is>
           <t>prefiltro</t>
         </is>
@@ -6609,7 +6377,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">BIO-009: Avian influenza outbreaks: evaluating the efficacy of cleaning and disinfection  | BIO-046: Risk Areas for Influenza A(H5) Environmental Contamination in Live Bird Markets, | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar | F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de </t>
+          <t xml:space="preserve">BIO-009: Avian influenza outbreaks: evaluating the efficacy of cleaning and disinfection  | BIO-046: Risk Areas for Influenza A(H5) Environmental Contamination in Live Bird Markets, | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de </t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -6657,7 +6425,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>F1;E7</t>
+          <t>D3;E7</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -6696,7 +6464,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar | C5: Avian Influenza: informacion general y medidas de prevencion (ficha tecnica ofic | C28: Gripe aviar y otras gripes de origen zoonotico (nota descriptiva)</t>
+          <t>F2: INFORME EPIDEMIOLÓGICO: Vigilancia de expuestos a influenza aviar | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | C5: Avian Influenza: informacion general y medidas de prevencion (ficha tecnica ofic | C28: Gripe aviar y otras gripes de origen zoonotico (nota descriptiva)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -6725,7 +6493,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>C11: Carbon dioxide and nitrogen infused compressed air foam for depopulation of cage | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar</t>
+          <t>C11: Carbon dioxide and nitrogen infused compressed air foam for depopulation of cage | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -6783,7 +6551,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BIO-068: Risk factors for avian influenza in Danish poultry and wild birds during the epi | F1: PLAN DE CONTINGENCIA VERSIÓN 6.0 Influenza Aviar | C18: Mortality levels and production indicators for suspicion of highly pathogenic av | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | E7: Procedimiento P-PP-VE-006 – Contingencia de Influenza Aviar</t>
+          <t>BIO-068: Risk factors for avian influenza in Danish poultry and wild birds during the epi | D3: Plan de Contingencia Influenza Aviar (IA), Version 6.0 | C18: Mortality levels and production indicators for suspicion of highly pathogenic av | C31: Alerta epidemiologica: Casos humanos de influenza aviar A(H5N1) en la Region de  | E7: Procedimiento P-PP-VE-006 – Contingencia de Influenza Aviar</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>

</xml_diff>